<commit_message>
[B8-B9] Add DG-5F-S $7,500 price scenario to roi.xlsx; reflect in analysis and B4 proposal with R-configuration trial budget; update knowledge, plan, progress (fact-check skipped by user)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/case/roi.xlsx
+++ b/case/roi.xlsx
@@ -29,7 +29,7 @@
     <numFmt numFmtId="169" formatCode="+0%;-0%;0%"/>
     <numFmt numFmtId="170" formatCode="0.0000"/>
   </numFmts>
-  <fonts count="7">
+  <fonts count="8">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -58,6 +58,12 @@
     <font>
       <b val="1"/>
       <color rgb="000000FF"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color theme="1"/>
+      <sz val="11"/>
     </font>
   </fonts>
   <fills count="5">
@@ -109,7 +115,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="42">
+  <cellXfs count="48">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -182,6 +188,16 @@
     </xf>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="170" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="2" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -556,7 +572,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H34"/>
+  <dimension ref="A1:H51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -1072,13 +1088,390 @@
         </is>
       </c>
     </row>
+    <row r="36">
+      <c r="A36" s="3" t="inlineStr">
+        <is>
+          <t>6. 손 단가 시나리오 - $23,000(제품 DB, 기본) 대 $7,500(RLWRLD 블로그) (B8, 민감도 시트 8절 링크)</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="48" customHeight="1">
+      <c r="A37" s="42" t="inlineStr">
+        <is>
+          <t>손 단가는 견적 전까지 헤드라인에 반영하지 않는다. 두 값 모두 공식 견적이 아니며(추정) Tesollo 공식 견적으로 확정한다. 아래는 '이 단가라면 이렇다'는 민감도 비교이고, 기본 시나리오(위 1절)는 $23,000 그대로다. 연동 = 통합비가 하드웨어(손 포함)에 비례(현 모델), 비연동 = 통합비를 $23,000 기준 금액으로 고정.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="45" customHeight="1">
+      <c r="A38" s="4" t="inlineStr">
+        <is>
+          <t>손 교체 시나리오</t>
+        </is>
+      </c>
+      <c r="B38" s="4" t="inlineStr">
+        <is>
+          <t>총 투자비 $23,000 (원)</t>
+        </is>
+      </c>
+      <c r="C38" s="4" t="inlineStr">
+        <is>
+          <t>총 투자비 $7,500 연동 (원)</t>
+        </is>
+      </c>
+      <c r="D38" s="4" t="inlineStr">
+        <is>
+          <t>총 투자비 $7,500 비연동 (원)</t>
+        </is>
+      </c>
+      <c r="E38" s="4" t="inlineStr">
+        <is>
+          <t>회수 $23,000 (년)</t>
+        </is>
+      </c>
+      <c r="F38" s="4" t="inlineStr">
+        <is>
+          <t>회수 $7,500 연동 (년)</t>
+        </is>
+      </c>
+      <c r="G38" s="4" t="inlineStr">
+        <is>
+          <t>회수 $7,500 비연동 (년)</t>
+        </is>
+      </c>
+      <c r="H38" s="4" t="inlineStr">
+        <is>
+          <t>회수 단축 연동 (년)</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>낙관 (f1, 20%)</t>
+        </is>
+      </c>
+      <c r="B39" s="9">
+        <f>'민감도'!B106</f>
+        <v/>
+      </c>
+      <c r="C39" s="9">
+        <f>'민감도'!C106</f>
+        <v/>
+      </c>
+      <c r="D39" s="9">
+        <f>'민감도'!C107</f>
+        <v/>
+      </c>
+      <c r="E39" s="10">
+        <f>'민감도'!B111</f>
+        <v/>
+      </c>
+      <c r="F39" s="10">
+        <f>'민감도'!C111</f>
+        <v/>
+      </c>
+      <c r="G39" s="10">
+        <f>'민감도'!C113</f>
+        <v/>
+      </c>
+      <c r="H39" s="10">
+        <f>'민감도'!D111</f>
+        <v/>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>기본 (f2, 20%)</t>
+        </is>
+      </c>
+      <c r="B40" s="9">
+        <f>'민감도'!E106</f>
+        <v/>
+      </c>
+      <c r="C40" s="9">
+        <f>'민감도'!F106</f>
+        <v/>
+      </c>
+      <c r="D40" s="9">
+        <f>'민감도'!F107</f>
+        <v/>
+      </c>
+      <c r="E40" s="10">
+        <f>'민감도'!E111</f>
+        <v/>
+      </c>
+      <c r="F40" s="10">
+        <f>'민감도'!F111</f>
+        <v/>
+      </c>
+      <c r="G40" s="10">
+        <f>'민감도'!F113</f>
+        <v/>
+      </c>
+      <c r="H40" s="10">
+        <f>'민감도'!G111</f>
+        <v/>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>보수 (f2, 100%)</t>
+        </is>
+      </c>
+      <c r="B41" s="9">
+        <f>'민감도'!H106</f>
+        <v/>
+      </c>
+      <c r="C41" s="9">
+        <f>'민감도'!I106</f>
+        <v/>
+      </c>
+      <c r="D41" s="9">
+        <f>'민감도'!I107</f>
+        <v/>
+      </c>
+      <c r="E41" s="10">
+        <f>'민감도'!H111</f>
+        <v/>
+      </c>
+      <c r="F41" s="10">
+        <f>'민감도'!I111</f>
+        <v/>
+      </c>
+      <c r="G41" s="10">
+        <f>'민감도'!I113</f>
+        <v/>
+      </c>
+      <c r="H41" s="10">
+        <f>'민감도'!J111</f>
+        <v/>
+      </c>
+    </row>
+    <row r="43" ht="45" customHeight="1">
+      <c r="A43" s="4" t="inlineStr">
+        <is>
+          <t>손 교체 시나리오</t>
+        </is>
+      </c>
+      <c r="B43" s="4" t="inlineStr">
+        <is>
+          <t>5년 NPV $23,000 (원)</t>
+        </is>
+      </c>
+      <c r="C43" s="4" t="inlineStr">
+        <is>
+          <t>5년 NPV $7,500 연동 (원)</t>
+        </is>
+      </c>
+      <c r="D43" s="4" t="inlineStr">
+        <is>
+          <t>5년 NPV $7,500 비연동 (원)</t>
+        </is>
+      </c>
+      <c r="E43" s="4" t="inlineStr">
+        <is>
+          <t>손 소모비 $23,000 (원/년)</t>
+        </is>
+      </c>
+      <c r="F43" s="4" t="inlineStr">
+        <is>
+          <t>손 소모비 $7,500 (원/년)</t>
+        </is>
+      </c>
+      <c r="G43" s="4" t="inlineStr">
+        <is>
+          <t>NPV 개선 연동 (원)</t>
+        </is>
+      </c>
+      <c r="H43" s="4" t="inlineStr">
+        <is>
+          <t>NPV 개선 비연동 (원)</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>낙관 (f1, 20%)</t>
+        </is>
+      </c>
+      <c r="B44" s="9">
+        <f>'민감도'!B112</f>
+        <v/>
+      </c>
+      <c r="C44" s="9">
+        <f>'민감도'!C112</f>
+        <v/>
+      </c>
+      <c r="D44" s="9">
+        <f>'민감도'!C114</f>
+        <v/>
+      </c>
+      <c r="E44" s="9">
+        <f>'민감도'!B108</f>
+        <v/>
+      </c>
+      <c r="F44" s="9">
+        <f>'민감도'!C108</f>
+        <v/>
+      </c>
+      <c r="G44" s="9">
+        <f>'민감도'!D112</f>
+        <v/>
+      </c>
+      <c r="H44" s="9">
+        <f>D44-B44</f>
+        <v/>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>기본 (f2, 20%)</t>
+        </is>
+      </c>
+      <c r="B45" s="9">
+        <f>'민감도'!E112</f>
+        <v/>
+      </c>
+      <c r="C45" s="9">
+        <f>'민감도'!F112</f>
+        <v/>
+      </c>
+      <c r="D45" s="9">
+        <f>'민감도'!F114</f>
+        <v/>
+      </c>
+      <c r="E45" s="9">
+        <f>'민감도'!E108</f>
+        <v/>
+      </c>
+      <c r="F45" s="9">
+        <f>'민감도'!F108</f>
+        <v/>
+      </c>
+      <c r="G45" s="9">
+        <f>'민감도'!G112</f>
+        <v/>
+      </c>
+      <c r="H45" s="9">
+        <f>D45-B45</f>
+        <v/>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>보수 (f2, 100%)</t>
+        </is>
+      </c>
+      <c r="B46" s="9">
+        <f>'민감도'!H112</f>
+        <v/>
+      </c>
+      <c r="C46" s="9">
+        <f>'민감도'!I112</f>
+        <v/>
+      </c>
+      <c r="D46" s="9">
+        <f>'민감도'!I114</f>
+        <v/>
+      </c>
+      <c r="E46" s="9">
+        <f>'민감도'!H108</f>
+        <v/>
+      </c>
+      <c r="F46" s="9">
+        <f>'민감도'!I108</f>
+        <v/>
+      </c>
+      <c r="G46" s="9">
+        <f>'민감도'!J112</f>
+        <v/>
+      </c>
+      <c r="H46" s="9">
+        <f>D46-B46</f>
+        <v/>
+      </c>
+    </row>
+    <row r="48" ht="45" customHeight="1">
+      <c r="A48" s="4" t="inlineStr">
+        <is>
+          <t>손 대 그리퍼(Hand-E $7,250, 추정) 하드웨어 비교</t>
+        </is>
+      </c>
+      <c r="B48" s="4" t="inlineStr">
+        <is>
+          <t>손 1개 단가비 $23,000 (배)</t>
+        </is>
+      </c>
+      <c r="C48" s="4" t="inlineStr">
+        <is>
+          <t>손 1개 단가비 $7,500 (배)</t>
+        </is>
+      </c>
+      <c r="D48" s="4" t="inlineStr">
+        <is>
+          <t>셀 하드웨어비 $23,000 (배)</t>
+        </is>
+      </c>
+      <c r="E48" s="4" t="inlineStr">
+        <is>
+          <t>셀 하드웨어비 $7,500 (배)</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" ht="45" customHeight="1">
+      <c r="A49" s="2" t="inlineStr">
+        <is>
+          <t>손 구성 대 그리퍼 구성 (단가비: 손 1개/Hand-E 1개, 셀: 손 구성/그리퍼 구성 하드웨어 합계)</t>
+        </is>
+      </c>
+      <c r="B49" s="43">
+        <f>'가정'!$D$49/'가정'!$D$76</f>
+        <v/>
+      </c>
+      <c r="C49" s="43">
+        <f>'가정'!$D$87/'가정'!$D$76</f>
+        <v/>
+      </c>
+      <c r="D49" s="43">
+        <f>'계산'!$C$23/'계산'!$C$36</f>
+        <v/>
+      </c>
+      <c r="E49" s="43">
+        <f>'민감도'!F101/'계산'!$C$36</f>
+        <v/>
+      </c>
+    </row>
+    <row r="50" ht="32" customHeight="1">
+      <c r="A50" s="2">
+        <f>"→ 손 1개 단가가 그리퍼의 "&amp;TEXT(B49,"0.0")&amp;"배에서 "&amp;TEXT(C49,"0.00")&amp;"배로 바뀐다($23,000 대 $7,500, Hand-E $7,250 추정). 셀 하드웨어는 "&amp;TEXT(D49,"0.00")&amp;"배에서 "&amp;TEXT(E49,"0.00")&amp;"배다."</f>
+        <v/>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>검산 시트 D절(B8) 불일치 건수 (0이어야 함)</t>
+        </is>
+      </c>
+      <c r="F51" s="30">
+        <f>'검산'!$C$83</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="8">
+  <mergeCells count="10">
+    <mergeCell ref="A50:H50"/>
     <mergeCell ref="A30:H30"/>
     <mergeCell ref="A29:H29"/>
     <mergeCell ref="A2:H2"/>
     <mergeCell ref="A28:H28"/>
     <mergeCell ref="A33:H33"/>
+    <mergeCell ref="A37:H37"/>
     <mergeCell ref="A32:H32"/>
     <mergeCell ref="A31:H31"/>
     <mergeCell ref="A34:H34"/>
@@ -1093,7 +1486,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G85"/>
+  <dimension ref="A1:G87"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -2612,7 +3005,7 @@
       </c>
       <c r="F49" s="2" t="inlineStr">
         <is>
-          <t>case/analysis.md 7.3절 [32], research/q7 6-1절. https://humanoid.guide/product/dg-5f-s/ (reference/hardware--tesollo-dg5f-s.md). 제품 DB 표기, 공식가 미확인</t>
+          <t>case/analysis.md 7.3절 [32], research/q7 6-1절. https://humanoid.guide/product/dg-5f-s/ (reference/hardware--tesollo-dg5f-s.md). 제품 DB 표기 $23,000(기본 시나리오 유지). 충돌값: RLWRLD 블로그 약 $7,500(research/q9-allhandsup.md 7절, reference/hardware--allhandsup-blog-part2.md)은 D87에 시나리오로 입력. 둘 다 공식 견적 아님 - 추정. Tesollo 공식 견적으로 확정 전까지 헤드라인에 반영하지 않음. 이 셀 하나가 투자비·통합비·손 소모비를 모두 구동</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
@@ -3808,6 +4201,54 @@
         </is>
       </c>
       <c r="G85" t="inlineStr">
+        <is>
+          <t>추정</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="15" t="inlineStr">
+        <is>
+          <t>8. 손 단가 시나리오 (B8, 기본 계산에는 쓰이지 않고 민감도 시트 8절 비교에만 사용)</t>
+        </is>
+      </c>
+      <c r="B86" s="16" t="n"/>
+      <c r="C86" s="16" t="n"/>
+      <c r="D86" s="16" t="n"/>
+      <c r="E86" s="16" t="n"/>
+      <c r="F86" s="16" t="n"/>
+      <c r="G86" s="16" t="n"/>
+    </row>
+    <row r="87" ht="62" customHeight="1">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>A74</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>손 단가 시나리오</t>
+        </is>
+      </c>
+      <c r="C87" s="2" t="inlineStr">
+        <is>
+          <t>다관절 손(20-DoF) 단가 - 대안 (RLWRLD 블로그 표기)</t>
+        </is>
+      </c>
+      <c r="D87" s="21" t="n">
+        <v>7500</v>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>USD/개</t>
+        </is>
+      </c>
+      <c r="F87" s="2" t="inlineStr">
+        <is>
+          <t>research/q9-allhandsup.md 7절 1행, reference/hardware--allhandsup-blog-part2.md (RLWRLD 블로그 'approximately $7,500 per hand'). 제품 DB($23,000, D49)와 충돌하며 둘 다 공식 견적이 아니므로 추정. Tesollo 공식 견적(구성·수량·환율)으로 확정할 것. 확정 전 헤드라인 미반영</t>
+        </is>
+      </c>
+      <c r="G87" t="inlineStr">
         <is>
           <t>추정</t>
         </is>
@@ -4186,7 +4627,6 @@
           <t>촉각 센서 소계 (USD)</t>
         </is>
       </c>
-      <c r="B20" t="inlineStr"/>
       <c r="C20" s="13">
         <f>'가정'!$D$51*'가정'!$D$52</f>
         <v/>
@@ -4198,7 +4638,6 @@
           <t>카메라 소계 (USD)</t>
         </is>
       </c>
-      <c r="B21" t="inlineStr"/>
       <c r="C21" s="13">
         <f>'가정'!$D$53*'가정'!$D$54</f>
         <v/>
@@ -4394,7 +4833,6 @@
           <t>연 정비비 하한 (원/년, 전체 그리퍼)</t>
         </is>
       </c>
-      <c r="B35" t="inlineStr"/>
       <c r="C35" s="13">
         <f>IF(ISNUMBER('가정'!$D$81),'가정'!$D$77*'가정'!$D$81/C33,"가격 미입력")</f>
         <v/>
@@ -4596,7 +5034,6 @@
           <t>속도비</t>
         </is>
       </c>
-      <c r="B41" t="inlineStr"/>
       <c r="C41" s="25">
         <f>'가정'!$D$14</f>
         <v/>
@@ -4662,7 +5099,6 @@
           <t>교대 수</t>
         </is>
       </c>
-      <c r="B42" t="inlineStr"/>
       <c r="C42" s="30">
         <f>'가정'!$D$9</f>
         <v/>
@@ -4979,7 +5415,6 @@
           <t>연 인건비/인 (원)</t>
         </is>
       </c>
-      <c r="B47" t="inlineStr"/>
       <c r="C47" s="13">
         <f>IF(ISNUMBER(C45),C45,INDEX($C$13:$E$13,C40))</f>
         <v/>
@@ -6015,7 +6450,6 @@
           <t>5년 내 회수?</t>
         </is>
       </c>
-      <c r="B60" t="inlineStr"/>
       <c r="C60" s="11">
         <f>IF(C58&gt;=0,"예","아니오")</f>
         <v/>
@@ -6309,10 +6743,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I89"/>
+  <dimension ref="A1:J116"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="44" customWidth="1" min="1" max="1"/>
+    <col width="48" customWidth="1" min="1" max="1"/>
     <col width="15" customWidth="1" min="2" max="2"/>
     <col width="15" customWidth="1" min="3" max="3"/>
     <col width="15" customWidth="1" min="4" max="4"/>
@@ -6320,6 +6754,9 @@
     <col width="15" customWidth="1" min="6" max="6"/>
     <col width="15" customWidth="1" min="7" max="7"/>
     <col width="15" customWidth="1" min="8" max="8"/>
+    <col width="15" customWidth="1" min="9" max="9"/>
+    <col width="15" customWidth="1" min="10" max="10"/>
+    <col width="15" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -7601,17 +8038,940 @@
         <v/>
       </c>
     </row>
+    <row r="92">
+      <c r="A92" s="3" t="inlineStr">
+        <is>
+          <t>8. 손 단가 시나리오 - $23,000(제품 DB, 기본) 대 $7,500(RLWRLD 블로그) (B8)</t>
+        </is>
+      </c>
+    </row>
+    <row r="93" ht="62" customHeight="1">
+      <c r="A93" s="2" t="inlineStr">
+        <is>
+          <t>손 단가는 가정 시트 D49(기본)와 D87(대안) 입력 셀 하나씩이며 투자비, 통합비, 손 소모비가 모두 이 값을 따른다. 팔·시스템 유지보수는 '손 제외 하드웨어' 기준이라 손 단가와 무관하다. 통합비는 현 모델이 하드웨어 합계(손 포함)에 비례하므로 '연동'이 현 모델 방식이고, '비연동'은 통합비를 $23,000 기준 금액으로 고정한 값이다. 둘 다 공식 견적이 아니므로 헤드라인에는 반영하지 않는다(추정).</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="29" t="inlineStr">
+        <is>
+          <t>손 교체 시나리오</t>
+        </is>
+      </c>
+      <c r="B94" s="29" t="inlineStr">
+        <is>
+          <t>낙관 (f1, 20%)</t>
+        </is>
+      </c>
+      <c r="C94" s="29" t="n"/>
+      <c r="D94" s="29" t="n"/>
+      <c r="E94" s="29" t="inlineStr">
+        <is>
+          <t>기본 (f2, 20%)</t>
+        </is>
+      </c>
+      <c r="F94" s="29" t="n"/>
+      <c r="G94" s="29" t="n"/>
+      <c r="H94" s="29" t="inlineStr">
+        <is>
+          <t>보수 (f2, 100%)</t>
+        </is>
+      </c>
+      <c r="I94" s="29" t="n"/>
+      <c r="J94" s="29" t="n"/>
+    </row>
+    <row r="95">
+      <c r="A95" s="29" t="inlineStr">
+        <is>
+          <t>항목 \ 손 단가</t>
+        </is>
+      </c>
+      <c r="B95" s="29" t="inlineStr">
+        <is>
+          <t>$23,000 (D49)</t>
+        </is>
+      </c>
+      <c r="C95" s="29" t="inlineStr">
+        <is>
+          <t>$7,500 (D87)</t>
+        </is>
+      </c>
+      <c r="D95" s="29" t="inlineStr">
+        <is>
+          <t>차이 (7,500-23,000)</t>
+        </is>
+      </c>
+      <c r="E95" s="29" t="inlineStr">
+        <is>
+          <t>$23,000 (D49)</t>
+        </is>
+      </c>
+      <c r="F95" s="29" t="inlineStr">
+        <is>
+          <t>$7,500 (D87)</t>
+        </is>
+      </c>
+      <c r="G95" s="29" t="inlineStr">
+        <is>
+          <t>차이 (7,500-23,000)</t>
+        </is>
+      </c>
+      <c r="H95" s="29" t="inlineStr">
+        <is>
+          <t>$23,000 (D49)</t>
+        </is>
+      </c>
+      <c r="I95" s="29" t="inlineStr">
+        <is>
+          <t>$7,500 (D87)</t>
+        </is>
+      </c>
+      <c r="J95" s="29" t="inlineStr">
+        <is>
+          <t>차이 (7,500-23,000)</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>f: 손 1개당 연 교체 횟수 (2교대 기준)</t>
+        </is>
+      </c>
+      <c r="B96" s="12">
+        <f>'가정'!$D$64</f>
+        <v/>
+      </c>
+      <c r="C96" s="12">
+        <f>'가정'!$D$64</f>
+        <v/>
+      </c>
+      <c r="D96" s="13" t="n"/>
+      <c r="E96" s="12">
+        <f>'가정'!$D$66</f>
+        <v/>
+      </c>
+      <c r="F96" s="12">
+        <f>'가정'!$D$66</f>
+        <v/>
+      </c>
+      <c r="G96" s="13" t="n"/>
+      <c r="H96" s="12">
+        <f>'가정'!$D$68</f>
+        <v/>
+      </c>
+      <c r="I96" s="12">
+        <f>'가정'!$D$68</f>
+        <v/>
+      </c>
+      <c r="J96" s="13" t="n"/>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>교체당 비용 비율 (손 가격 대비)</t>
+        </is>
+      </c>
+      <c r="B97" s="25">
+        <f>'가정'!$D$65</f>
+        <v/>
+      </c>
+      <c r="C97" s="25">
+        <f>'가정'!$D$65</f>
+        <v/>
+      </c>
+      <c r="D97" s="13" t="n"/>
+      <c r="E97" s="25">
+        <f>'가정'!$D$67</f>
+        <v/>
+      </c>
+      <c r="F97" s="25">
+        <f>'가정'!$D$67</f>
+        <v/>
+      </c>
+      <c r="G97" s="13" t="n"/>
+      <c r="H97" s="25">
+        <f>'가정'!$D$69</f>
+        <v/>
+      </c>
+      <c r="I97" s="25">
+        <f>'가정'!$D$69</f>
+        <v/>
+      </c>
+      <c r="J97" s="13" t="n"/>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>손 단가 (USD/개)</t>
+        </is>
+      </c>
+      <c r="B98" s="13">
+        <f>'가정'!$D$49</f>
+        <v/>
+      </c>
+      <c r="C98" s="13">
+        <f>'가정'!$D$87</f>
+        <v/>
+      </c>
+      <c r="D98" s="13">
+        <f>IF(AND(ISNUMBER(B98),ISNUMBER(C98)),C98-B98,"-")</f>
+        <v/>
+      </c>
+      <c r="E98" s="13">
+        <f>'가정'!$D$49</f>
+        <v/>
+      </c>
+      <c r="F98" s="13">
+        <f>'가정'!$D$87</f>
+        <v/>
+      </c>
+      <c r="G98" s="13">
+        <f>IF(AND(ISNUMBER(E98),ISNUMBER(F98)),F98-E98,"-")</f>
+        <v/>
+      </c>
+      <c r="H98" s="13">
+        <f>'가정'!$D$49</f>
+        <v/>
+      </c>
+      <c r="I98" s="13">
+        <f>'가정'!$D$87</f>
+        <v/>
+      </c>
+      <c r="J98" s="13">
+        <f>IF(AND(ISNUMBER(H98),ISNUMBER(I98)),I98-H98,"-")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>손 투자비 (USD, 손 개수분)</t>
+        </is>
+      </c>
+      <c r="B99" s="13">
+        <f>B98*'가정'!$D$50</f>
+        <v/>
+      </c>
+      <c r="C99" s="13">
+        <f>C98*'가정'!$D$50</f>
+        <v/>
+      </c>
+      <c r="D99" s="13">
+        <f>IF(AND(ISNUMBER(B99),ISNUMBER(C99)),C99-B99,"-")</f>
+        <v/>
+      </c>
+      <c r="E99" s="13">
+        <f>E98*'가정'!$D$50</f>
+        <v/>
+      </c>
+      <c r="F99" s="13">
+        <f>F98*'가정'!$D$50</f>
+        <v/>
+      </c>
+      <c r="G99" s="13">
+        <f>IF(AND(ISNUMBER(E99),ISNUMBER(F99)),F99-E99,"-")</f>
+        <v/>
+      </c>
+      <c r="H99" s="13">
+        <f>H98*'가정'!$D$50</f>
+        <v/>
+      </c>
+      <c r="I99" s="13">
+        <f>I98*'가정'!$D$50</f>
+        <v/>
+      </c>
+      <c r="J99" s="13">
+        <f>IF(AND(ISNUMBER(H99),ISNUMBER(I99)),I99-H99,"-")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>손 외 하드웨어 (USD, 팔+센서+카메라+지그+PC)</t>
+        </is>
+      </c>
+      <c r="B100" s="13">
+        <f>'계산'!$C$18+'계산'!$C$22</f>
+        <v/>
+      </c>
+      <c r="C100" s="13">
+        <f>'계산'!$C$18+'계산'!$C$22</f>
+        <v/>
+      </c>
+      <c r="D100" s="13">
+        <f>IF(AND(ISNUMBER(B100),ISNUMBER(C100)),C100-B100,"-")</f>
+        <v/>
+      </c>
+      <c r="E100" s="13">
+        <f>'계산'!$C$18+'계산'!$C$22</f>
+        <v/>
+      </c>
+      <c r="F100" s="13">
+        <f>'계산'!$C$18+'계산'!$C$22</f>
+        <v/>
+      </c>
+      <c r="G100" s="13">
+        <f>IF(AND(ISNUMBER(E100),ISNUMBER(F100)),F100-E100,"-")</f>
+        <v/>
+      </c>
+      <c r="H100" s="13">
+        <f>'계산'!$C$18+'계산'!$C$22</f>
+        <v/>
+      </c>
+      <c r="I100" s="13">
+        <f>'계산'!$C$18+'계산'!$C$22</f>
+        <v/>
+      </c>
+      <c r="J100" s="13">
+        <f>IF(AND(ISNUMBER(H100),ISNUMBER(I100)),I100-H100,"-")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>하드웨어 합계 (USD)</t>
+        </is>
+      </c>
+      <c r="B101" s="13">
+        <f>B99+B100</f>
+        <v/>
+      </c>
+      <c r="C101" s="13">
+        <f>C99+C100</f>
+        <v/>
+      </c>
+      <c r="D101" s="13">
+        <f>IF(AND(ISNUMBER(B101),ISNUMBER(C101)),C101-B101,"-")</f>
+        <v/>
+      </c>
+      <c r="E101" s="13">
+        <f>E99+E100</f>
+        <v/>
+      </c>
+      <c r="F101" s="13">
+        <f>F99+F100</f>
+        <v/>
+      </c>
+      <c r="G101" s="13">
+        <f>IF(AND(ISNUMBER(E101),ISNUMBER(F101)),F101-E101,"-")</f>
+        <v/>
+      </c>
+      <c r="H101" s="13">
+        <f>H99+H100</f>
+        <v/>
+      </c>
+      <c r="I101" s="13">
+        <f>I99+I100</f>
+        <v/>
+      </c>
+      <c r="J101" s="13">
+        <f>IF(AND(ISNUMBER(H101),ISNUMBER(I101)),I101-H101,"-")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>통합비 (USD) - 연동 (하드웨어 비례, 현 모델)</t>
+        </is>
+      </c>
+      <c r="B102" s="13">
+        <f>B101*'가정'!$D$57</f>
+        <v/>
+      </c>
+      <c r="C102" s="13">
+        <f>C101*'가정'!$D$57</f>
+        <v/>
+      </c>
+      <c r="D102" s="13">
+        <f>IF(AND(ISNUMBER(B102),ISNUMBER(C102)),C102-B102,"-")</f>
+        <v/>
+      </c>
+      <c r="E102" s="13">
+        <f>E101*'가정'!$D$57</f>
+        <v/>
+      </c>
+      <c r="F102" s="13">
+        <f>F101*'가정'!$D$57</f>
+        <v/>
+      </c>
+      <c r="G102" s="13">
+        <f>IF(AND(ISNUMBER(E102),ISNUMBER(F102)),F102-E102,"-")</f>
+        <v/>
+      </c>
+      <c r="H102" s="13">
+        <f>H101*'가정'!$D$57</f>
+        <v/>
+      </c>
+      <c r="I102" s="13">
+        <f>I101*'가정'!$D$57</f>
+        <v/>
+      </c>
+      <c r="J102" s="13">
+        <f>IF(AND(ISNUMBER(H102),ISNUMBER(I102)),I102-H102,"-")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>통합비 (USD) - 비연동 ($23,000 기준 고정)</t>
+        </is>
+      </c>
+      <c r="B103" s="13">
+        <f>(B100+'가정'!$D$49*'가정'!$D$50)*'가정'!$D$57</f>
+        <v/>
+      </c>
+      <c r="C103" s="13">
+        <f>(C100+'가정'!$D$49*'가정'!$D$50)*'가정'!$D$57</f>
+        <v/>
+      </c>
+      <c r="D103" s="13">
+        <f>IF(AND(ISNUMBER(B103),ISNUMBER(C103)),C103-B103,"-")</f>
+        <v/>
+      </c>
+      <c r="E103" s="13">
+        <f>(E100+'가정'!$D$49*'가정'!$D$50)*'가정'!$D$57</f>
+        <v/>
+      </c>
+      <c r="F103" s="13">
+        <f>(F100+'가정'!$D$49*'가정'!$D$50)*'가정'!$D$57</f>
+        <v/>
+      </c>
+      <c r="G103" s="13">
+        <f>IF(AND(ISNUMBER(E103),ISNUMBER(F103)),F103-E103,"-")</f>
+        <v/>
+      </c>
+      <c r="H103" s="13">
+        <f>(H100+'가정'!$D$49*'가정'!$D$50)*'가정'!$D$57</f>
+        <v/>
+      </c>
+      <c r="I103" s="13">
+        <f>(I100+'가정'!$D$49*'가정'!$D$50)*'가정'!$D$57</f>
+        <v/>
+      </c>
+      <c r="J103" s="13">
+        <f>IF(AND(ISNUMBER(H103),ISNUMBER(I103)),I103-H103,"-")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>총 투자비 (USD) - 연동</t>
+        </is>
+      </c>
+      <c r="B104" s="13">
+        <f>B101+B102</f>
+        <v/>
+      </c>
+      <c r="C104" s="13">
+        <f>C101+C102</f>
+        <v/>
+      </c>
+      <c r="D104" s="13">
+        <f>IF(AND(ISNUMBER(B104),ISNUMBER(C104)),C104-B104,"-")</f>
+        <v/>
+      </c>
+      <c r="E104" s="13">
+        <f>E101+E102</f>
+        <v/>
+      </c>
+      <c r="F104" s="13">
+        <f>F101+F102</f>
+        <v/>
+      </c>
+      <c r="G104" s="13">
+        <f>IF(AND(ISNUMBER(E104),ISNUMBER(F104)),F104-E104,"-")</f>
+        <v/>
+      </c>
+      <c r="H104" s="13">
+        <f>H101+H102</f>
+        <v/>
+      </c>
+      <c r="I104" s="13">
+        <f>I101+I102</f>
+        <v/>
+      </c>
+      <c r="J104" s="13">
+        <f>IF(AND(ISNUMBER(H104),ISNUMBER(I104)),I104-H104,"-")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>총 투자비 (USD) - 비연동</t>
+        </is>
+      </c>
+      <c r="B105" s="13">
+        <f>B101+B103</f>
+        <v/>
+      </c>
+      <c r="C105" s="13">
+        <f>C101+C103</f>
+        <v/>
+      </c>
+      <c r="D105" s="13">
+        <f>IF(AND(ISNUMBER(B105),ISNUMBER(C105)),C105-B105,"-")</f>
+        <v/>
+      </c>
+      <c r="E105" s="13">
+        <f>E101+E103</f>
+        <v/>
+      </c>
+      <c r="F105" s="13">
+        <f>F101+F103</f>
+        <v/>
+      </c>
+      <c r="G105" s="13">
+        <f>IF(AND(ISNUMBER(E105),ISNUMBER(F105)),F105-E105,"-")</f>
+        <v/>
+      </c>
+      <c r="H105" s="13">
+        <f>H101+H103</f>
+        <v/>
+      </c>
+      <c r="I105" s="13">
+        <f>I101+I103</f>
+        <v/>
+      </c>
+      <c r="J105" s="13">
+        <f>IF(AND(ISNUMBER(H105),ISNUMBER(I105)),I105-H105,"-")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>총 투자비 (원) - 연동</t>
+        </is>
+      </c>
+      <c r="B106" s="13">
+        <f>B104*'가정'!$D$46+'가정'!$D$58</f>
+        <v/>
+      </c>
+      <c r="C106" s="13">
+        <f>C104*'가정'!$D$46+'가정'!$D$58</f>
+        <v/>
+      </c>
+      <c r="D106" s="13">
+        <f>IF(AND(ISNUMBER(B106),ISNUMBER(C106)),C106-B106,"-")</f>
+        <v/>
+      </c>
+      <c r="E106" s="13">
+        <f>E104*'가정'!$D$46+'가정'!$D$58</f>
+        <v/>
+      </c>
+      <c r="F106" s="13">
+        <f>F104*'가정'!$D$46+'가정'!$D$58</f>
+        <v/>
+      </c>
+      <c r="G106" s="13">
+        <f>IF(AND(ISNUMBER(E106),ISNUMBER(F106)),F106-E106,"-")</f>
+        <v/>
+      </c>
+      <c r="H106" s="13">
+        <f>H104*'가정'!$D$46+'가정'!$D$58</f>
+        <v/>
+      </c>
+      <c r="I106" s="13">
+        <f>I104*'가정'!$D$46+'가정'!$D$58</f>
+        <v/>
+      </c>
+      <c r="J106" s="13">
+        <f>IF(AND(ISNUMBER(H106),ISNUMBER(I106)),I106-H106,"-")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>총 투자비 (원) - 비연동</t>
+        </is>
+      </c>
+      <c r="B107" s="13">
+        <f>B105*'가정'!$D$46+'가정'!$D$58</f>
+        <v/>
+      </c>
+      <c r="C107" s="13">
+        <f>C105*'가정'!$D$46+'가정'!$D$58</f>
+        <v/>
+      </c>
+      <c r="D107" s="13">
+        <f>IF(AND(ISNUMBER(B107),ISNUMBER(C107)),C107-B107,"-")</f>
+        <v/>
+      </c>
+      <c r="E107" s="13">
+        <f>E105*'가정'!$D$46+'가정'!$D$58</f>
+        <v/>
+      </c>
+      <c r="F107" s="13">
+        <f>F105*'가정'!$D$46+'가정'!$D$58</f>
+        <v/>
+      </c>
+      <c r="G107" s="13">
+        <f>IF(AND(ISNUMBER(E107),ISNUMBER(F107)),F107-E107,"-")</f>
+        <v/>
+      </c>
+      <c r="H107" s="13">
+        <f>H105*'가정'!$D$46+'가정'!$D$58</f>
+        <v/>
+      </c>
+      <c r="I107" s="13">
+        <f>I105*'가정'!$D$46+'가정'!$D$58</f>
+        <v/>
+      </c>
+      <c r="J107" s="13">
+        <f>IF(AND(ISNUMBER(H107),ISNUMBER(I107)),I107-H107,"-")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>손 소모비 (원/년)</t>
+        </is>
+      </c>
+      <c r="B108" s="13">
+        <f>'가정'!$D$50*B96*'계산'!$C$42/'가정'!$D$63*B97*B98*'가정'!$D$46</f>
+        <v/>
+      </c>
+      <c r="C108" s="13">
+        <f>'가정'!$D$50*C96*'계산'!$C$42/'가정'!$D$63*C97*C98*'가정'!$D$46</f>
+        <v/>
+      </c>
+      <c r="D108" s="13">
+        <f>IF(AND(ISNUMBER(B108),ISNUMBER(C108)),C108-B108,"-")</f>
+        <v/>
+      </c>
+      <c r="E108" s="13">
+        <f>'가정'!$D$50*E96*'계산'!$C$42/'가정'!$D$63*E97*E98*'가정'!$D$46</f>
+        <v/>
+      </c>
+      <c r="F108" s="13">
+        <f>'가정'!$D$50*F96*'계산'!$C$42/'가정'!$D$63*F97*F98*'가정'!$D$46</f>
+        <v/>
+      </c>
+      <c r="G108" s="13">
+        <f>IF(AND(ISNUMBER(E108),ISNUMBER(F108)),F108-E108,"-")</f>
+        <v/>
+      </c>
+      <c r="H108" s="13">
+        <f>'가정'!$D$50*H96*'계산'!$C$42/'가정'!$D$63*H97*H98*'가정'!$D$46</f>
+        <v/>
+      </c>
+      <c r="I108" s="13">
+        <f>'가정'!$D$50*I96*'계산'!$C$42/'가정'!$D$63*I97*I98*'가정'!$D$46</f>
+        <v/>
+      </c>
+      <c r="J108" s="13">
+        <f>IF(AND(ISNUMBER(H108),ISNUMBER(I108)),I108-H108,"-")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>연간 운영비 (원)</t>
+        </is>
+      </c>
+      <c r="B109" s="13">
+        <f>'계산'!$C$50+B108+'계산'!$C$53</f>
+        <v/>
+      </c>
+      <c r="C109" s="13">
+        <f>'계산'!$C$50+C108+'계산'!$C$53</f>
+        <v/>
+      </c>
+      <c r="D109" s="13">
+        <f>IF(AND(ISNUMBER(B109),ISNUMBER(C109)),C109-B109,"-")</f>
+        <v/>
+      </c>
+      <c r="E109" s="13">
+        <f>'계산'!$C$50+E108+'계산'!$C$53</f>
+        <v/>
+      </c>
+      <c r="F109" s="13">
+        <f>'계산'!$C$50+F108+'계산'!$C$53</f>
+        <v/>
+      </c>
+      <c r="G109" s="13">
+        <f>IF(AND(ISNUMBER(E109),ISNUMBER(F109)),F109-E109,"-")</f>
+        <v/>
+      </c>
+      <c r="H109" s="13">
+        <f>'계산'!$C$50+H108+'계산'!$C$53</f>
+        <v/>
+      </c>
+      <c r="I109" s="13">
+        <f>'계산'!$C$50+I108+'계산'!$C$53</f>
+        <v/>
+      </c>
+      <c r="J109" s="13">
+        <f>IF(AND(ISNUMBER(H109),ISNUMBER(I109)),I109-H109,"-")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>연간 순효과 (원)</t>
+        </is>
+      </c>
+      <c r="B110" s="13">
+        <f>'계산'!$C$49-B109</f>
+        <v/>
+      </c>
+      <c r="C110" s="13">
+        <f>'계산'!$C$49-C109</f>
+        <v/>
+      </c>
+      <c r="D110" s="13">
+        <f>IF(AND(ISNUMBER(B110),ISNUMBER(C110)),C110-B110,"-")</f>
+        <v/>
+      </c>
+      <c r="E110" s="13">
+        <f>'계산'!$C$49-E109</f>
+        <v/>
+      </c>
+      <c r="F110" s="13">
+        <f>'계산'!$C$49-F109</f>
+        <v/>
+      </c>
+      <c r="G110" s="13">
+        <f>IF(AND(ISNUMBER(E110),ISNUMBER(F110)),F110-E110,"-")</f>
+        <v/>
+      </c>
+      <c r="H110" s="13">
+        <f>'계산'!$C$49-H109</f>
+        <v/>
+      </c>
+      <c r="I110" s="13">
+        <f>'계산'!$C$49-I109</f>
+        <v/>
+      </c>
+      <c r="J110" s="13">
+        <f>IF(AND(ISNUMBER(H110),ISNUMBER(I110)),I110-H110,"-")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="44" t="inlineStr">
+        <is>
+          <t>단순 회수 기간 (년) - 연동</t>
+        </is>
+      </c>
+      <c r="B111" s="45">
+        <f>IF(B110&gt;0,B106/B110,"회수 불가")</f>
+        <v/>
+      </c>
+      <c r="C111" s="45">
+        <f>IF(C110&gt;0,C106/C110,"회수 불가")</f>
+        <v/>
+      </c>
+      <c r="D111" s="46">
+        <f>IF(AND(ISNUMBER(B111),ISNUMBER(C111)),C111-B111,"-")</f>
+        <v/>
+      </c>
+      <c r="E111" s="45">
+        <f>IF(E110&gt;0,E106/E110,"회수 불가")</f>
+        <v/>
+      </c>
+      <c r="F111" s="45">
+        <f>IF(F110&gt;0,F106/F110,"회수 불가")</f>
+        <v/>
+      </c>
+      <c r="G111" s="46">
+        <f>IF(AND(ISNUMBER(E111),ISNUMBER(F111)),F111-E111,"-")</f>
+        <v/>
+      </c>
+      <c r="H111" s="45">
+        <f>IF(H110&gt;0,H106/H110,"회수 불가")</f>
+        <v/>
+      </c>
+      <c r="I111" s="45">
+        <f>IF(I110&gt;0,I106/I110,"회수 불가")</f>
+        <v/>
+      </c>
+      <c r="J111" s="46">
+        <f>IF(AND(ISNUMBER(H111),ISNUMBER(I111)),I111-H111,"-")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" s="44" t="inlineStr">
+        <is>
+          <t>5년 NPV (원) - 연동</t>
+        </is>
+      </c>
+      <c r="B112" s="47">
+        <f>-B106+NPV('가정'!$D$83,B110,B110,B110,B110,B110)</f>
+        <v/>
+      </c>
+      <c r="C112" s="47">
+        <f>-C106+NPV('가정'!$D$83,C110,C110,C110,C110,C110)</f>
+        <v/>
+      </c>
+      <c r="D112" s="47">
+        <f>IF(AND(ISNUMBER(B112),ISNUMBER(C112)),C112-B112,"-")</f>
+        <v/>
+      </c>
+      <c r="E112" s="47">
+        <f>-E106+NPV('가정'!$D$83,E110,E110,E110,E110,E110)</f>
+        <v/>
+      </c>
+      <c r="F112" s="47">
+        <f>-F106+NPV('가정'!$D$83,F110,F110,F110,F110,F110)</f>
+        <v/>
+      </c>
+      <c r="G112" s="47">
+        <f>IF(AND(ISNUMBER(E112),ISNUMBER(F112)),F112-E112,"-")</f>
+        <v/>
+      </c>
+      <c r="H112" s="47">
+        <f>-H106+NPV('가정'!$D$83,H110,H110,H110,H110,H110)</f>
+        <v/>
+      </c>
+      <c r="I112" s="47">
+        <f>-I106+NPV('가정'!$D$83,I110,I110,I110,I110,I110)</f>
+        <v/>
+      </c>
+      <c r="J112" s="47">
+        <f>IF(AND(ISNUMBER(H112),ISNUMBER(I112)),I112-H112,"-")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" s="44" t="inlineStr">
+        <is>
+          <t>단순 회수 기간 (년) - 비연동</t>
+        </is>
+      </c>
+      <c r="B113" s="45">
+        <f>IF(B110&gt;0,B107/B110,"회수 불가")</f>
+        <v/>
+      </c>
+      <c r="C113" s="45">
+        <f>IF(C110&gt;0,C107/C110,"회수 불가")</f>
+        <v/>
+      </c>
+      <c r="D113" s="46">
+        <f>IF(AND(ISNUMBER(B113),ISNUMBER(C113)),C113-B113,"-")</f>
+        <v/>
+      </c>
+      <c r="E113" s="45">
+        <f>IF(E110&gt;0,E107/E110,"회수 불가")</f>
+        <v/>
+      </c>
+      <c r="F113" s="45">
+        <f>IF(F110&gt;0,F107/F110,"회수 불가")</f>
+        <v/>
+      </c>
+      <c r="G113" s="46">
+        <f>IF(AND(ISNUMBER(E113),ISNUMBER(F113)),F113-E113,"-")</f>
+        <v/>
+      </c>
+      <c r="H113" s="45">
+        <f>IF(H110&gt;0,H107/H110,"회수 불가")</f>
+        <v/>
+      </c>
+      <c r="I113" s="45">
+        <f>IF(I110&gt;0,I107/I110,"회수 불가")</f>
+        <v/>
+      </c>
+      <c r="J113" s="46">
+        <f>IF(AND(ISNUMBER(H113),ISNUMBER(I113)),I113-H113,"-")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" s="44" t="inlineStr">
+        <is>
+          <t>5년 NPV (원) - 비연동</t>
+        </is>
+      </c>
+      <c r="B114" s="47">
+        <f>-B107+NPV('가정'!$D$83,B110,B110,B110,B110,B110)</f>
+        <v/>
+      </c>
+      <c r="C114" s="47">
+        <f>-C107+NPV('가정'!$D$83,C110,C110,C110,C110,C110)</f>
+        <v/>
+      </c>
+      <c r="D114" s="47">
+        <f>IF(AND(ISNUMBER(B114),ISNUMBER(C114)),C114-B114,"-")</f>
+        <v/>
+      </c>
+      <c r="E114" s="47">
+        <f>-E107+NPV('가정'!$D$83,E110,E110,E110,E110,E110)</f>
+        <v/>
+      </c>
+      <c r="F114" s="47">
+        <f>-F107+NPV('가정'!$D$83,F110,F110,F110,F110,F110)</f>
+        <v/>
+      </c>
+      <c r="G114" s="47">
+        <f>IF(AND(ISNUMBER(E114),ISNUMBER(F114)),F114-E114,"-")</f>
+        <v/>
+      </c>
+      <c r="H114" s="47">
+        <f>-H107+NPV('가정'!$D$83,H110,H110,H110,H110,H110)</f>
+        <v/>
+      </c>
+      <c r="I114" s="47">
+        <f>-I107+NPV('가정'!$D$83,I110,I110,I110,I110,I110)</f>
+        <v/>
+      </c>
+      <c r="J114" s="47">
+        <f>IF(AND(ISNUMBER(H114),ISNUMBER(I114)),I114-H114,"-")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="115" ht="32" customHeight="1">
+      <c r="A115" s="2" t="inlineStr">
+        <is>
+          <t>기준 확인: 기본(f2·20%) $23,000 열의 회수·NPV가 계산 시트 기본 열과 같은가 (가정 D7=2일 때만 해당)</t>
+        </is>
+      </c>
+      <c r="E115">
+        <f>IF('가정'!$D$7=2,IF(AND(ABS(E112-'계산'!C59)&lt;1,ABS(E111-'계산'!C56)&lt;0.0005),"일치","불일치"),"선택 아님")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="116" ht="32" customHeight="1">
+      <c r="A116" s="2" t="inlineStr">
+        <is>
+          <t>손 단가가 5년 NPV에 주는 폭 (기본 f2·20%, 연동, 백만 원) 대 1절 최대 변수 폭</t>
+        </is>
+      </c>
+      <c r="E116" s="13">
+        <f>ABS(G112)/1000000</f>
+        <v/>
+      </c>
+      <c r="F116">
+        <f>"1절 최대 폭 "&amp;TEXT(MAX($F$9:$F$17),"#,##0")&amp;" 백만 원"</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="9">
+  <mergeCells count="13">
     <mergeCell ref="A74:H74"/>
     <mergeCell ref="A67:H67"/>
+    <mergeCell ref="A93:J93"/>
     <mergeCell ref="A2:I2"/>
+    <mergeCell ref="B94:D94"/>
+    <mergeCell ref="H94:J94"/>
     <mergeCell ref="A82:H82"/>
     <mergeCell ref="A60:H60"/>
     <mergeCell ref="A41:H41"/>
     <mergeCell ref="A5:E5"/>
     <mergeCell ref="A6:E6"/>
     <mergeCell ref="A22:H22"/>
+    <mergeCell ref="E94:G94"/>
   </mergeCells>
   <conditionalFormatting sqref="B24:D28">
     <cfRule type="expression" priority="1" dxfId="0">
@@ -7658,7 +9018,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H42"/>
+  <dimension ref="A1:H88"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="54" customWidth="1" min="1" max="1"/>
@@ -8853,6 +10213,1352 @@
         <v/>
       </c>
     </row>
+    <row r="44">
+      <c r="A44" s="14" t="inlineStr">
+        <is>
+          <t>D. 손 단가 시나리오 (B8) - 민감도 시트 8절 vs Python 독립 계산, 허용오차 년 0.0005 / 원 1,000</t>
+        </is>
+      </c>
+      <c r="H44" s="2" t="n"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="2" t="inlineStr">
+        <is>
+          <t>낙관 f1·20% $23,000 연동: 총 투자비</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>원</t>
+        </is>
+      </c>
+      <c r="C45" s="13" t="n">
+        <v>395584000</v>
+      </c>
+      <c r="D45" s="13">
+        <f>'민감도'!B106</f>
+        <v/>
+      </c>
+      <c r="E45" s="13">
+        <f>D45-C45</f>
+        <v/>
+      </c>
+      <c r="F45">
+        <f>IF(ABS(E45)&lt;=1000,"일치","불일치")</f>
+        <v/>
+      </c>
+      <c r="H45" s="2" t="inlineStr">
+        <is>
+          <t>신규(B8), 문서 값 없음</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="2" t="inlineStr">
+        <is>
+          <t>낙관 f1·20% $23,000 연동: 회수 기간</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>년</t>
+        </is>
+      </c>
+      <c r="C46" s="41" t="n">
+        <v>3.919160833925549</v>
+      </c>
+      <c r="D46" s="41">
+        <f>'민감도'!B111</f>
+        <v/>
+      </c>
+      <c r="E46" s="41">
+        <f>IF(AND(ISNUMBER(C46),ISNUMBER(D46)),D46-C46,IF(C46=D46,0,999))</f>
+        <v/>
+      </c>
+      <c r="F46">
+        <f>IF(ABS(E46)&lt;=0.0005,"일치","불일치")</f>
+        <v/>
+      </c>
+      <c r="H46" s="2" t="inlineStr">
+        <is>
+          <t>신규(B8), 문서 값 없음</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="2" t="inlineStr">
+        <is>
+          <t>낙관 f1·20% $23,000 연동: 5년 NPV</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>원</t>
+        </is>
+      </c>
+      <c r="C47" s="13" t="n">
+        <v>7423754.526233673</v>
+      </c>
+      <c r="D47" s="13">
+        <f>'민감도'!B112</f>
+        <v/>
+      </c>
+      <c r="E47" s="13">
+        <f>D47-C47</f>
+        <v/>
+      </c>
+      <c r="F47">
+        <f>IF(ABS(E47)&lt;=1000,"일치","불일치")</f>
+        <v/>
+      </c>
+      <c r="H47" s="2" t="inlineStr">
+        <is>
+          <t>신규(B8), 문서 값 없음</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="2" t="inlineStr">
+        <is>
+          <t>낙관 f1·20% $23,000: 손 소모비</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>원/년</t>
+        </is>
+      </c>
+      <c r="C48" s="13" t="n">
+        <v>12880000</v>
+      </c>
+      <c r="D48" s="13">
+        <f>'민감도'!B108</f>
+        <v/>
+      </c>
+      <c r="E48" s="13">
+        <f>D48-C48</f>
+        <v/>
+      </c>
+      <c r="F48">
+        <f>IF(ABS(E48)&lt;=1000,"일치","불일치")</f>
+        <v/>
+      </c>
+      <c r="H48" s="2" t="inlineStr">
+        <is>
+          <t>신규(B8), 문서 값 없음</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="2" t="inlineStr">
+        <is>
+          <t>낙관 f1·20% $7,500 연동: 총 투자비</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>원</t>
+        </is>
+      </c>
+      <c r="C49" s="13" t="n">
+        <v>308784000</v>
+      </c>
+      <c r="D49" s="13">
+        <f>'민감도'!C106</f>
+        <v/>
+      </c>
+      <c r="E49" s="13">
+        <f>D49-C49</f>
+        <v/>
+      </c>
+      <c r="F49">
+        <f>IF(ABS(E49)&lt;=1000,"일치","불일치")</f>
+        <v/>
+      </c>
+      <c r="H49" s="2" t="inlineStr">
+        <is>
+          <t>신규(B8), 문서 값 없음</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="inlineStr">
+        <is>
+          <t>낙관 f1·20% $7,500 연동: 회수 기간</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>년</t>
+        </is>
+      </c>
+      <c r="C50" s="41" t="n">
+        <v>2.816963768031659</v>
+      </c>
+      <c r="D50" s="41">
+        <f>'민감도'!C111</f>
+        <v/>
+      </c>
+      <c r="E50" s="41">
+        <f>IF(AND(ISNUMBER(C50),ISNUMBER(D50)),D50-C50,IF(C50=D50,0,999))</f>
+        <v/>
+      </c>
+      <c r="F50">
+        <f>IF(ABS(E50)&lt;=0.0005,"일치","불일치")</f>
+        <v/>
+      </c>
+      <c r="H50" s="2" t="inlineStr">
+        <is>
+          <t>신규(B8), 문서 값 없음</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="2" t="inlineStr">
+        <is>
+          <t>낙관 f1·20% $7,500 연동: 5년 NPV</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>원</t>
+        </is>
+      </c>
+      <c r="C51" s="13" t="n">
+        <v>128880477.6480715</v>
+      </c>
+      <c r="D51" s="13">
+        <f>'민감도'!C112</f>
+        <v/>
+      </c>
+      <c r="E51" s="13">
+        <f>D51-C51</f>
+        <v/>
+      </c>
+      <c r="F51">
+        <f>IF(ABS(E51)&lt;=1000,"일치","불일치")</f>
+        <v/>
+      </c>
+      <c r="H51" s="2" t="inlineStr">
+        <is>
+          <t>신규(B8), 문서 값 없음</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="2" t="inlineStr">
+        <is>
+          <t>낙관 f1·20% $7,500 비연동: 총 투자비</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>원</t>
+        </is>
+      </c>
+      <c r="C52" s="13" t="n">
+        <v>352184000</v>
+      </c>
+      <c r="D52" s="13">
+        <f>'민감도'!C107</f>
+        <v/>
+      </c>
+      <c r="E52" s="13">
+        <f>D52-C52</f>
+        <v/>
+      </c>
+      <c r="F52">
+        <f>IF(ABS(E52)&lt;=1000,"일치","불일치")</f>
+        <v/>
+      </c>
+      <c r="H52" s="2" t="inlineStr">
+        <is>
+          <t>신규(B8), 문서 값 없음</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="2" t="inlineStr">
+        <is>
+          <t>낙관 f1·20% $7,500 비연동: 회수 기간</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>년</t>
+        </is>
+      </c>
+      <c r="C53" s="41" t="n">
+        <v>3.212891755014709</v>
+      </c>
+      <c r="D53" s="41">
+        <f>'민감도'!C113</f>
+        <v/>
+      </c>
+      <c r="E53" s="41">
+        <f>IF(AND(ISNUMBER(C53),ISNUMBER(D53)),D53-C53,IF(C53=D53,0,999))</f>
+        <v/>
+      </c>
+      <c r="F53">
+        <f>IF(ABS(E53)&lt;=0.0005,"일치","불일치")</f>
+        <v/>
+      </c>
+      <c r="H53" s="2" t="inlineStr">
+        <is>
+          <t>신규(B8), 문서 값 없음</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="2" t="inlineStr">
+        <is>
+          <t>낙관 f1·20% $7,500 비연동: 5년 NPV</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>원</t>
+        </is>
+      </c>
+      <c r="C54" s="13" t="n">
+        <v>85480477.64807147</v>
+      </c>
+      <c r="D54" s="13">
+        <f>'민감도'!C114</f>
+        <v/>
+      </c>
+      <c r="E54" s="13">
+        <f>D54-C54</f>
+        <v/>
+      </c>
+      <c r="F54">
+        <f>IF(ABS(E54)&lt;=1000,"일치","불일치")</f>
+        <v/>
+      </c>
+      <c r="H54" s="2" t="inlineStr">
+        <is>
+          <t>신규(B8), 문서 값 없음</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="2" t="inlineStr">
+        <is>
+          <t>낙관 f1·20% $7,500: 손 소모비</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>원/년</t>
+        </is>
+      </c>
+      <c r="C55" s="13" t="n">
+        <v>4200000</v>
+      </c>
+      <c r="D55" s="13">
+        <f>'민감도'!C108</f>
+        <v/>
+      </c>
+      <c r="E55" s="13">
+        <f>D55-C55</f>
+        <v/>
+      </c>
+      <c r="F55">
+        <f>IF(ABS(E55)&lt;=1000,"일치","불일치")</f>
+        <v/>
+      </c>
+      <c r="H55" s="2" t="inlineStr">
+        <is>
+          <t>신규(B8), 문서 값 없음</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="2" t="inlineStr">
+        <is>
+          <t>기본 f2·20% $23,000 연동: 총 투자비</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>원</t>
+        </is>
+      </c>
+      <c r="C56" s="13" t="n">
+        <v>395584000</v>
+      </c>
+      <c r="D56" s="13">
+        <f>'민감도'!E106</f>
+        <v/>
+      </c>
+      <c r="E56" s="13">
+        <f>D56-C56</f>
+        <v/>
+      </c>
+      <c r="F56">
+        <f>IF(ABS(E56)&lt;=1000,"일치","불일치")</f>
+        <v/>
+      </c>
+      <c r="H56" s="2" t="inlineStr">
+        <is>
+          <t>신규(B8), 문서 값 없음</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="2" t="inlineStr">
+        <is>
+          <t>기본 f2·20% $23,000 연동: 회수 기간</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>년</t>
+        </is>
+      </c>
+      <c r="C57" s="41" t="n">
+        <v>4.49241935886812</v>
+      </c>
+      <c r="D57" s="41">
+        <f>'민감도'!E111</f>
+        <v/>
+      </c>
+      <c r="E57" s="41">
+        <f>IF(AND(ISNUMBER(C57),ISNUMBER(D57)),D57-C57,IF(C57=D57,0,999))</f>
+        <v/>
+      </c>
+      <c r="F57">
+        <f>IF(ABS(E57)&lt;=0.0005,"일치","불일치")</f>
+        <v/>
+      </c>
+      <c r="H57" s="2" t="inlineStr">
+        <is>
+          <t>신규(B8), 문서 값 없음</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="2" t="inlineStr">
+        <is>
+          <t>기본 f2·20% $23,000 연동: 5년 NPV</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>원</t>
+        </is>
+      </c>
+      <c r="C58" s="13" t="n">
+        <v>-44002350.75133204</v>
+      </c>
+      <c r="D58" s="13">
+        <f>'민감도'!E112</f>
+        <v/>
+      </c>
+      <c r="E58" s="13">
+        <f>D58-C58</f>
+        <v/>
+      </c>
+      <c r="F58">
+        <f>IF(ABS(E58)&lt;=1000,"일치","불일치")</f>
+        <v/>
+      </c>
+      <c r="H58" s="2" t="inlineStr">
+        <is>
+          <t>신규(B8), 문서 값 없음</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="2" t="inlineStr">
+        <is>
+          <t>기본 f2·20% $23,000: 손 소모비</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>원/년</t>
+        </is>
+      </c>
+      <c r="C59" s="13" t="n">
+        <v>25760000</v>
+      </c>
+      <c r="D59" s="13">
+        <f>'민감도'!E108</f>
+        <v/>
+      </c>
+      <c r="E59" s="13">
+        <f>D59-C59</f>
+        <v/>
+      </c>
+      <c r="F59">
+        <f>IF(ABS(E59)&lt;=1000,"일치","불일치")</f>
+        <v/>
+      </c>
+      <c r="H59" s="2" t="inlineStr">
+        <is>
+          <t>신규(B8), 문서 값 없음</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="2" t="inlineStr">
+        <is>
+          <t>기본 f2·20% $7,500 연동: 총 투자비</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>원</t>
+        </is>
+      </c>
+      <c r="C60" s="13" t="n">
+        <v>308784000</v>
+      </c>
+      <c r="D60" s="13">
+        <f>'민감도'!F106</f>
+        <v/>
+      </c>
+      <c r="E60" s="13">
+        <f>D60-C60</f>
+        <v/>
+      </c>
+      <c r="F60">
+        <f>IF(ABS(E60)&lt;=1000,"일치","불일치")</f>
+        <v/>
+      </c>
+      <c r="H60" s="2" t="inlineStr">
+        <is>
+          <t>신규(B8), 문서 값 없음</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="2" t="inlineStr">
+        <is>
+          <t>기본 f2·20% $7,500 연동: 회수 기간</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>년</t>
+        </is>
+      </c>
+      <c r="C61" s="41" t="n">
+        <v>2.929197772302259</v>
+      </c>
+      <c r="D61" s="41">
+        <f>'민감도'!F111</f>
+        <v/>
+      </c>
+      <c r="E61" s="41">
+        <f>IF(AND(ISNUMBER(C61),ISNUMBER(D61)),D61-C61,IF(C61=D61,0,999))</f>
+        <v/>
+      </c>
+      <c r="F61">
+        <f>IF(ABS(E61)&lt;=0.0005,"일치","불일치")</f>
+        <v/>
+      </c>
+      <c r="H61" s="2" t="inlineStr">
+        <is>
+          <t>신규(B8), 문서 값 없음</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="2" t="inlineStr">
+        <is>
+          <t>기본 f2·20% $7,500 연동: 5년 NPV</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>원</t>
+        </is>
+      </c>
+      <c r="C62" s="13" t="n">
+        <v>112111095.4923435</v>
+      </c>
+      <c r="D62" s="13">
+        <f>'민감도'!F112</f>
+        <v/>
+      </c>
+      <c r="E62" s="13">
+        <f>D62-C62</f>
+        <v/>
+      </c>
+      <c r="F62">
+        <f>IF(ABS(E62)&lt;=1000,"일치","불일치")</f>
+        <v/>
+      </c>
+      <c r="H62" s="2" t="inlineStr">
+        <is>
+          <t>신규(B8), 문서 값 없음</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="2" t="inlineStr">
+        <is>
+          <t>기본 f2·20% $7,500 비연동: 총 투자비</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>원</t>
+        </is>
+      </c>
+      <c r="C63" s="13" t="n">
+        <v>352184000</v>
+      </c>
+      <c r="D63" s="13">
+        <f>'민감도'!F107</f>
+        <v/>
+      </c>
+      <c r="E63" s="13">
+        <f>D63-C63</f>
+        <v/>
+      </c>
+      <c r="F63">
+        <f>IF(ABS(E63)&lt;=1000,"일치","불일치")</f>
+        <v/>
+      </c>
+      <c r="H63" s="2" t="inlineStr">
+        <is>
+          <t>신규(B8), 문서 값 없음</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="2" t="inlineStr">
+        <is>
+          <t>기본 f2·20% $7,500 비연동: 회수 기간</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>년</t>
+        </is>
+      </c>
+      <c r="C64" s="41" t="n">
+        <v>3.340900397172454</v>
+      </c>
+      <c r="D64" s="41">
+        <f>'민감도'!F113</f>
+        <v/>
+      </c>
+      <c r="E64" s="41">
+        <f>IF(AND(ISNUMBER(C64),ISNUMBER(D64)),D64-C64,IF(C64=D64,0,999))</f>
+        <v/>
+      </c>
+      <c r="F64">
+        <f>IF(ABS(E64)&lt;=0.0005,"일치","불일치")</f>
+        <v/>
+      </c>
+      <c r="H64" s="2" t="inlineStr">
+        <is>
+          <t>신규(B8), 문서 값 없음</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="2" t="inlineStr">
+        <is>
+          <t>기본 f2·20% $7,500 비연동: 5년 NPV</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>원</t>
+        </is>
+      </c>
+      <c r="C65" s="13" t="n">
+        <v>68711095.49234349</v>
+      </c>
+      <c r="D65" s="13">
+        <f>'민감도'!F114</f>
+        <v/>
+      </c>
+      <c r="E65" s="13">
+        <f>D65-C65</f>
+        <v/>
+      </c>
+      <c r="F65">
+        <f>IF(ABS(E65)&lt;=1000,"일치","불일치")</f>
+        <v/>
+      </c>
+      <c r="H65" s="2" t="inlineStr">
+        <is>
+          <t>신규(B8), 문서 값 없음</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="2" t="inlineStr">
+        <is>
+          <t>기본 f2·20% $7,500: 손 소모비</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>원/년</t>
+        </is>
+      </c>
+      <c r="C66" s="13" t="n">
+        <v>8400000</v>
+      </c>
+      <c r="D66" s="13">
+        <f>'민감도'!F108</f>
+        <v/>
+      </c>
+      <c r="E66" s="13">
+        <f>D66-C66</f>
+        <v/>
+      </c>
+      <c r="F66">
+        <f>IF(ABS(E66)&lt;=1000,"일치","불일치")</f>
+        <v/>
+      </c>
+      <c r="H66" s="2" t="inlineStr">
+        <is>
+          <t>신규(B8), 문서 값 없음</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="2" t="inlineStr">
+        <is>
+          <t>보수 f2·100% $23,000 연동: 총 투자비</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>원</t>
+        </is>
+      </c>
+      <c r="C67" s="13" t="n">
+        <v>395584000</v>
+      </c>
+      <c r="D67" s="13">
+        <f>'민감도'!H106</f>
+        <v/>
+      </c>
+      <c r="E67" s="13">
+        <f>D67-C67</f>
+        <v/>
+      </c>
+      <c r="F67">
+        <f>IF(ABS(E67)&lt;=1000,"일치","불일치")</f>
+        <v/>
+      </c>
+      <c r="H67" s="2" t="inlineStr">
+        <is>
+          <t>신규(B8), 문서 값 없음</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="2" t="inlineStr">
+        <is>
+          <t>보수 f2·100% $23,000 연동: 회수 기간</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>년</t>
+        </is>
+      </c>
+      <c r="C68" s="41" t="inlineStr">
+        <is>
+          <t>회수 불가</t>
+        </is>
+      </c>
+      <c r="D68" s="41">
+        <f>'민감도'!H111</f>
+        <v/>
+      </c>
+      <c r="E68" s="41">
+        <f>IF(AND(ISNUMBER(C68),ISNUMBER(D68)),D68-C68,IF(C68=D68,0,999))</f>
+        <v/>
+      </c>
+      <c r="F68">
+        <f>IF(ABS(E68)&lt;=0.0005,"일치","불일치")</f>
+        <v/>
+      </c>
+      <c r="H68" s="2" t="inlineStr">
+        <is>
+          <t>신규(B8), 문서 값 없음</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="2" t="inlineStr">
+        <is>
+          <t>보수 f2·100% $23,000 연동: 5년 NPV</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>원</t>
+        </is>
+      </c>
+      <c r="C69" s="13" t="n">
+        <v>-455411192.9718579</v>
+      </c>
+      <c r="D69" s="13">
+        <f>'민감도'!H112</f>
+        <v/>
+      </c>
+      <c r="E69" s="13">
+        <f>D69-C69</f>
+        <v/>
+      </c>
+      <c r="F69">
+        <f>IF(ABS(E69)&lt;=1000,"일치","불일치")</f>
+        <v/>
+      </c>
+      <c r="H69" s="2" t="inlineStr">
+        <is>
+          <t>신규(B8), 문서 값 없음</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="2" t="inlineStr">
+        <is>
+          <t>보수 f2·100% $23,000: 손 소모비</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>원/년</t>
+        </is>
+      </c>
+      <c r="C70" s="13" t="n">
+        <v>128800000</v>
+      </c>
+      <c r="D70" s="13">
+        <f>'민감도'!H108</f>
+        <v/>
+      </c>
+      <c r="E70" s="13">
+        <f>D70-C70</f>
+        <v/>
+      </c>
+      <c r="F70">
+        <f>IF(ABS(E70)&lt;=1000,"일치","불일치")</f>
+        <v/>
+      </c>
+      <c r="H70" s="2" t="inlineStr">
+        <is>
+          <t>신규(B8), 문서 값 없음</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="2" t="inlineStr">
+        <is>
+          <t>보수 f2·100% $7,500 연동: 총 투자비</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>원</t>
+        </is>
+      </c>
+      <c r="C71" s="13" t="n">
+        <v>308784000</v>
+      </c>
+      <c r="D71" s="13">
+        <f>'민감도'!I106</f>
+        <v/>
+      </c>
+      <c r="E71" s="13">
+        <f>D71-C71</f>
+        <v/>
+      </c>
+      <c r="F71">
+        <f>IF(ABS(E71)&lt;=1000,"일치","불일치")</f>
+        <v/>
+      </c>
+      <c r="H71" s="2" t="inlineStr">
+        <is>
+          <t>신규(B8), 문서 값 없음</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="2" t="inlineStr">
+        <is>
+          <t>보수 f2·100% $7,500 연동: 회수 기간</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>년</t>
+        </is>
+      </c>
+      <c r="C72" s="41" t="n">
+        <v>4.299661057550559</v>
+      </c>
+      <c r="D72" s="41">
+        <f>'민감도'!I111</f>
+        <v/>
+      </c>
+      <c r="E72" s="41">
+        <f>IF(AND(ISNUMBER(C72),ISNUMBER(D72)),D72-C72,IF(C72=D72,0,999))</f>
+        <v/>
+      </c>
+      <c r="F72">
+        <f>IF(ABS(E72)&lt;=0.0005,"일치","불일치")</f>
+        <v/>
+      </c>
+      <c r="H72" s="2" t="inlineStr">
+        <is>
+          <t>신규(B8), 문서 값 없음</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="2" t="inlineStr">
+        <is>
+          <t>보수 f2·100% $7,500 연동: 5년 NPV</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>원</t>
+        </is>
+      </c>
+      <c r="C73" s="13" t="n">
+        <v>-22043961.75348014</v>
+      </c>
+      <c r="D73" s="13">
+        <f>'민감도'!I112</f>
+        <v/>
+      </c>
+      <c r="E73" s="13">
+        <f>D73-C73</f>
+        <v/>
+      </c>
+      <c r="F73">
+        <f>IF(ABS(E73)&lt;=1000,"일치","불일치")</f>
+        <v/>
+      </c>
+      <c r="H73" s="2" t="inlineStr">
+        <is>
+          <t>신규(B8), 문서 값 없음</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="2" t="inlineStr">
+        <is>
+          <t>보수 f2·100% $7,500 비연동: 총 투자비</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>원</t>
+        </is>
+      </c>
+      <c r="C74" s="13" t="n">
+        <v>352184000</v>
+      </c>
+      <c r="D74" s="13">
+        <f>'민감도'!I107</f>
+        <v/>
+      </c>
+      <c r="E74" s="13">
+        <f>D74-C74</f>
+        <v/>
+      </c>
+      <c r="F74">
+        <f>IF(ABS(E74)&lt;=1000,"일치","불일치")</f>
+        <v/>
+      </c>
+      <c r="H74" s="2" t="inlineStr">
+        <is>
+          <t>신규(B8), 문서 값 없음</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="2" t="inlineStr">
+        <is>
+          <t>보수 f2·100% $7,500 비연동: 회수 기간</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>년</t>
+        </is>
+      </c>
+      <c r="C75" s="41" t="n">
+        <v>4.903984111522573</v>
+      </c>
+      <c r="D75" s="41">
+        <f>'민감도'!I113</f>
+        <v/>
+      </c>
+      <c r="E75" s="41">
+        <f>IF(AND(ISNUMBER(C75),ISNUMBER(D75)),D75-C75,IF(C75=D75,0,999))</f>
+        <v/>
+      </c>
+      <c r="F75">
+        <f>IF(ABS(E75)&lt;=0.0005,"일치","불일치")</f>
+        <v/>
+      </c>
+      <c r="H75" s="2" t="inlineStr">
+        <is>
+          <t>신규(B8), 문서 값 없음</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="2" t="inlineStr">
+        <is>
+          <t>보수 f2·100% $7,500 비연동: 5년 NPV</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>원</t>
+        </is>
+      </c>
+      <c r="C76" s="13" t="n">
+        <v>-65443961.75348014</v>
+      </c>
+      <c r="D76" s="13">
+        <f>'민감도'!I114</f>
+        <v/>
+      </c>
+      <c r="E76" s="13">
+        <f>D76-C76</f>
+        <v/>
+      </c>
+      <c r="F76">
+        <f>IF(ABS(E76)&lt;=1000,"일치","불일치")</f>
+        <v/>
+      </c>
+      <c r="H76" s="2" t="inlineStr">
+        <is>
+          <t>신규(B8), 문서 값 없음</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="2" t="inlineStr">
+        <is>
+          <t>보수 f2·100% $7,500: 손 소모비</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>원/년</t>
+        </is>
+      </c>
+      <c r="C77" s="13" t="n">
+        <v>42000000</v>
+      </c>
+      <c r="D77" s="13">
+        <f>'민감도'!I108</f>
+        <v/>
+      </c>
+      <c r="E77" s="13">
+        <f>D77-C77</f>
+        <v/>
+      </c>
+      <c r="F77">
+        <f>IF(ABS(E77)&lt;=1000,"일치","불일치")</f>
+        <v/>
+      </c>
+      <c r="H77" s="2" t="inlineStr">
+        <is>
+          <t>신규(B8), 문서 값 없음</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="2" t="inlineStr">
+        <is>
+          <t>교차: 8절 기본 f2·20% $23,000 NPV - 계산 시트 C열 NPV (D7=2 기준)</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>원</t>
+        </is>
+      </c>
+      <c r="C78" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="D78" s="13">
+        <f>'민감도'!E112-'계산'!C59</f>
+        <v/>
+      </c>
+      <c r="E78" s="13">
+        <f>D78-C78</f>
+        <v/>
+      </c>
+      <c r="F78">
+        <f>IF(ABS(E78)&lt;=1000,"일치","불일치")</f>
+        <v/>
+      </c>
+      <c r="H78" s="2" t="inlineStr">
+        <is>
+          <t>8절이 기존 계산 열과 같은지 (기본 열은 가정 D7=2일 때)</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="2" t="inlineStr">
+        <is>
+          <t>교차: 8절 낙관 f1·20% $23,000 NPV - 계산 시트 F열 NPV (D7=2 기준)</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>원</t>
+        </is>
+      </c>
+      <c r="C79" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="D79" s="13">
+        <f>'민감도'!B112-'계산'!F59</f>
+        <v/>
+      </c>
+      <c r="E79" s="13">
+        <f>D79-C79</f>
+        <v/>
+      </c>
+      <c r="F79">
+        <f>IF(ABS(E79)&lt;=1000,"일치","불일치")</f>
+        <v/>
+      </c>
+      <c r="H79" s="2" t="inlineStr">
+        <is>
+          <t>8절이 기존 계산 열과 같은지 (기본 열은 가정 D7=2일 때)</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="2" t="inlineStr">
+        <is>
+          <t>교차: 8절 보수 f2·100% $23,000 NPV - 계산 시트 G열 NPV (D7=2 기준)</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>원</t>
+        </is>
+      </c>
+      <c r="C80" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="D80" s="13">
+        <f>'민감도'!H112-'계산'!G59</f>
+        <v/>
+      </c>
+      <c r="E80" s="13">
+        <f>D80-C80</f>
+        <v/>
+      </c>
+      <c r="F80">
+        <f>IF(ABS(E80)&lt;=1000,"일치","불일치")</f>
+        <v/>
+      </c>
+      <c r="H80" s="2" t="inlineStr">
+        <is>
+          <t>8절이 기존 계산 열과 같은지 (기본 열은 가정 D7=2일 때)</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="2" t="inlineStr">
+        <is>
+          <t>손 대 그리퍼 단가비 $23,000 / $7,500 (Python)</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>배</t>
+        </is>
+      </c>
+      <c r="C81" s="41" t="n">
+        <v>3.172413793103448</v>
+      </c>
+      <c r="D81" s="41">
+        <f>'요약'!B49</f>
+        <v/>
+      </c>
+      <c r="E81" s="41">
+        <f>D81-C81</f>
+        <v/>
+      </c>
+      <c r="F81">
+        <f>IF(ABS(E81)&lt;=0.0005,"일치","불일치")</f>
+        <v/>
+      </c>
+      <c r="H81" s="2" t="inlineStr">
+        <is>
+          <t>Q9/요청: 약 3.2배</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="2" t="inlineStr">
+        <is>
+          <t>손 대 그리퍼 단가비 $7,500 (Python)</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>배</t>
+        </is>
+      </c>
+      <c r="C82" s="41" t="n">
+        <v>1.03448275862069</v>
+      </c>
+      <c r="D82" s="41">
+        <f>'요약'!C49</f>
+        <v/>
+      </c>
+      <c r="E82" s="41">
+        <f>D82-C82</f>
+        <v/>
+      </c>
+      <c r="F82">
+        <f>IF(ABS(E82)&lt;=0.0005,"일치","불일치")</f>
+        <v/>
+      </c>
+      <c r="H82" s="2" t="inlineStr">
+        <is>
+          <t>Q9/요청: 약 1.03배</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="14" t="inlineStr">
+        <is>
+          <t>D절 불일치 건수 (0이어야 함)</t>
+        </is>
+      </c>
+      <c r="C83" s="3">
+        <f>COUNTIF(F45:F82,"불일치")</f>
+        <v/>
+      </c>
+      <c r="H83" s="2" t="n"/>
+    </row>
+    <row r="84">
+      <c r="A84" s="2" t="n"/>
+      <c r="H84" s="2" t="n"/>
+    </row>
+    <row r="85">
+      <c r="A85" s="14" t="inlineStr">
+        <is>
+          <t>E. Q9 근사(research/q9-allhandsup.md 7절)와 시트 계산 대조 - 차이는 이슈가 아니라 정의 차이</t>
+        </is>
+      </c>
+      <c r="H85" s="2" t="n"/>
+    </row>
+    <row r="86">
+      <c r="A86" s="2" t="inlineStr">
+        <is>
+          <t>Q9 기존 회수 약 4.5년 vs 시트 $23,000 기본(f2·20%)</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>년</t>
+        </is>
+      </c>
+      <c r="C86" s="25" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="D86" s="25">
+        <f>'민감도'!E111</f>
+        <v/>
+      </c>
+      <c r="E86" s="25">
+        <f>D86-C86</f>
+        <v/>
+      </c>
+      <c r="F86">
+        <f>IF(ABS(E86)&lt;=0.05,"일치","차이")</f>
+        <v/>
+      </c>
+      <c r="H86" s="2" t="inlineStr">
+        <is>
+          <t>Q9는 반올림 값(0.05년 허용)</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="2" t="inlineStr">
+        <is>
+          <t>Q9 근사 회수 약 3.3년 vs 시트 $7,500 비연동(손 투자만 감소)</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>년</t>
+        </is>
+      </c>
+      <c r="C87" s="25" t="n">
+        <v>3.3</v>
+      </c>
+      <c r="D87" s="25">
+        <f>'민감도'!F113</f>
+        <v/>
+      </c>
+      <c r="E87" s="25">
+        <f>D87-C87</f>
+        <v/>
+      </c>
+      <c r="F87">
+        <f>IF(ABS(E87)&lt;=0.05,"일치","차이")</f>
+        <v/>
+      </c>
+      <c r="H87" s="2" t="inlineStr">
+        <is>
+          <t>Q9식 = (395.6M-43.4M)/(88.06M+17.36M), 통합비 고정이므로 비연동과 같은 식</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="2" t="inlineStr">
+        <is>
+          <t>Q9 근사 회수 약 3.3년 vs 시트 $7,500 연동(현 모델 방식)</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>년</t>
+        </is>
+      </c>
+      <c r="C88" s="25" t="n">
+        <v>3.3</v>
+      </c>
+      <c r="D88" s="25">
+        <f>'민감도'!F111</f>
+        <v/>
+      </c>
+      <c r="E88" s="25">
+        <f>D88-C88</f>
+        <v/>
+      </c>
+      <c r="F88">
+        <f>IF(ABS(E88)&lt;=0.05,"일치","차이")</f>
+        <v/>
+      </c>
+      <c r="H88" s="2" t="inlineStr">
+        <is>
+          <t>원인: 현 모델의 통합비가 하드웨어(손 포함)에 비례(손 2개 x $15,500 x 100% 추가 감소 = 4,340만 원). Q9도 "연동되면 더 짧아진다"고 명시. 유지보수는 손 제외 기준이라 영향 없음</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A2:H2"/>

</xml_diff>